<commit_message>
Publish catalog 320d2 1.0.1
</commit_message>
<xml_diff>
--- a/catalog_cloud/catalogos/320d2.xlsx
+++ b/catalog_cloud/catalogos/320d2.xlsx
@@ -1,34 +1,292 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DESCARGAS\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24A2481-317C-4D93-84D9-5AA1183AAC3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="catalogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="catalogo" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="79">
+  <si>
+    <t>Código</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIFTER-VALVE |LEVANTAVÁLVULAS - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAMSHAFT GP |GRUPO DE ÁRBOL DE LEVAS - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">KEY-WOODRUFF |CHAVETA WOODRUFF - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROD |VARILLA - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLUG-SIDE |TAPÓN LATERAL - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOWEL |ESPIGA - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLUG |TAPÓN - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLUG-CORE |TAPÓN DE NÚCLEO - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOLT-SPECIAL |PERNO ESPECIAL - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUSHING-CAMSHAFT |BUJE DE ÁRBOL DE LEVAS - </t>
+  </si>
+  <si>
+    <t>BOLT |PERNO - (M8X1.25X16-MM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEAL-O-RING |SELLO ANULAR - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CYLINDER BLOCK AS |CONJUNTO DE BLOQUE DE CILINDRO - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOUSING AS |CONJUNTO DE CAJA - </t>
+  </si>
+  <si>
+    <t>BOLT |PERNO - (M6X1X10-MM)</t>
+  </si>
+  <si>
+    <t>TUBE AS-OIL JET |CONJUNTO DE TUBO DE CHORRO DE ACEITE - CONJUNTO DE TUBO DE CHORRO DE ACEITE</t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M8X1.25X20-MM)</t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M8X1.25X25-MM)</t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M10X1.5X65-MM)</t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M12X1.75X45-MM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOWEL |DOWEL| - </t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M8X1.25X65-MM)</t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M8X1.25X35-MM)</t>
+  </si>
+  <si>
+    <t>BOLT |BOLT| - (M8X1.25X16-MM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WASHER |WASHER| - </t>
+  </si>
+  <si>
+    <t>GEAR-CAMSHAFT |GEAR-CAMSHAFT| - (68-TEETH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GASKET-COVER |GASKET-COVER| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEAL |SEAL| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLUG |PLUG| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">KIT-COVER |KIT-COVER| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLATE |PLATE| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">COVER AS-FRONT |COVER AS-FRONT| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GASKET |GASKET| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">WASHER-THRUST |WASHER-THRUST| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HUB-IDLER GEAR |HUB-IDLER GEAR| - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GEAR-IDLER |GEAR-IDLER| - </t>
+  </si>
+  <si>
+    <t>4646253 </t>
+  </si>
+  <si>
+    <t>3889876 </t>
+  </si>
+  <si>
+    <t>0676135 </t>
+  </si>
+  <si>
+    <t>0676095 </t>
+  </si>
+  <si>
+    <t>0676043 </t>
+  </si>
+  <si>
+    <t>1850884 </t>
+  </si>
+  <si>
+    <t>2258858 </t>
+  </si>
+  <si>
+    <t>2327597 </t>
+  </si>
+  <si>
+    <t>2327599 </t>
+  </si>
+  <si>
+    <t>2765602 </t>
+  </si>
+  <si>
+    <t>2327596 </t>
+  </si>
+  <si>
+    <t>0676823 </t>
+  </si>
+  <si>
+    <t>2765600 </t>
+  </si>
+  <si>
+    <t>3706545 </t>
+  </si>
+  <si>
+    <t>2099219 </t>
+  </si>
+  <si>
+    <t>2321322 </t>
+  </si>
+  <si>
+    <t>2765603 </t>
+  </si>
+  <si>
+    <t>3311682 </t>
+  </si>
+  <si>
+    <t>2327449 </t>
+  </si>
+  <si>
+    <t>1004841 </t>
+  </si>
+  <si>
+    <t>3293796 </t>
+  </si>
+  <si>
+    <t>6I0217 </t>
+  </si>
+  <si>
+    <t>6I0645 </t>
+  </si>
+  <si>
+    <t>6I0650 </t>
+  </si>
+  <si>
+    <t>7C4616 </t>
+  </si>
+  <si>
+    <t>0676179 </t>
+  </si>
+  <si>
+    <t>1003751 </t>
+  </si>
+  <si>
+    <t>1013895 </t>
+  </si>
+  <si>
+    <t>1243815 </t>
+  </si>
+  <si>
+    <t>1331011 </t>
+  </si>
+  <si>
+    <t>2168634 </t>
+  </si>
+  <si>
+    <t>2773012 </t>
+  </si>
+  <si>
+    <t>2773013 </t>
+  </si>
+  <si>
+    <t>2774223 </t>
+  </si>
+  <si>
+    <t>2940286 </t>
+  </si>
+  <si>
+    <t>3460408 </t>
+  </si>
+  <si>
+    <t>2323657 </t>
+  </si>
+  <si>
+    <t>2258287 </t>
+  </si>
+  <si>
+    <t>2323666 </t>
+  </si>
+  <si>
+    <t>3240444 </t>
+  </si>
+  <si>
+    <t>3460407 </t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +305,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,36 +607,348 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B42"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="2" width="41.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Código</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PROD-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Producto de ejemplo</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>66</v>
+      </c>
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>67</v>
+      </c>
+      <c r="B31" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>